<commit_message>
fix(unit02): address Excel web review
</commit_message>
<xml_diff>
--- a/bus-math-nextjs/public/resources/unit02-lesson06-teacher.xlsx
+++ b/bus-math-nextjs/public/resources/unit02-lesson06-teacher.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>INDEX(Scenarios!$B$4:$B$6,MATCH(SelectedPeriod,Scenarios!$A$4:$A$6,0))</f>
+        <f>INDEX(Scenarios!$B$5:$F$7,MATCH(SelectedPeriod,Scenarios!$A$5:$A$7,0),ROW()-4)</f>
         <v/>
       </c>
       <c r="C5" s="4" t="n">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>INDEX(Scenarios!$C$4:$C$6,MATCH(SelectedPeriod,Scenarios!$A$4:$A$6,0))</f>
+        <f>INDEX(Scenarios!$B$5:$F$7,MATCH(SelectedPeriod,Scenarios!$A$5:$A$7,0),ROW()-4)</f>
         <v/>
       </c>
       <c r="C6" s="4" t="n">
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>INDEX(Scenarios!$D$4:$D$6,MATCH(SelectedPeriod,Scenarios!$A$4:$A$6,0))</f>
+        <f>INDEX(Scenarios!$B$5:$F$7,MATCH(SelectedPeriod,Scenarios!$A$5:$A$7,0),ROW()-4)</f>
         <v/>
       </c>
       <c r="C7" s="4" t="n">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>INDEX(Scenarios!$E$4:$E$6,MATCH(SelectedPeriod,Scenarios!$A$4:$A$6,0))</f>
+        <f>INDEX(Scenarios!$B$5:$F$7,MATCH(SelectedPeriod,Scenarios!$A$5:$A$7,0),ROW()-4)</f>
         <v/>
       </c>
       <c r="C8" s="4" t="n">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>INDEX(Scenarios!$F$4:$F$6,MATCH(SelectedPeriod,Scenarios!$A$4:$A$6,0))</f>
+        <f>INDEX(Scenarios!$B$5:$F$7,MATCH(SelectedPeriod,Scenarios!$A$5:$A$7,0),ROW()-4)</f>
         <v/>
       </c>
       <c r="C9" s="4" t="n">

</xml_diff>